<commit_message>
[UI] Cooking Item 필요한 재료 표시
</commit_message>
<xml_diff>
--- a/Sheets/ItemData.xlsx
+++ b/Sheets/ItemData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tfdkg\UnityProject\Farm\Sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0526128E-2A3F-470D-B933-6F44BF1A774B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19B7DA06-3B99-459D-8143-F3F142803D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-285" yWindow="30" windowWidth="28770" windowHeight="15450" activeTab="3" xr2:uid="{62B5C00F-698F-4EE8-88B3-1AC2C87E7411}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{62B5C00F-698F-4EE8-88B3-1AC2C87E7411}"/>
   </bookViews>
   <sheets>
     <sheet name="Objects" sheetId="6" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="182">
   <si>
     <t>Parsnip Seeds</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -673,10 +673,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>$Rep_ingredient$</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Recipe</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -774,6 +770,18 @@
   </si>
   <si>
     <t>$$Recipes$$</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OBJECTS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RECIPE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>$Req_ingredient$</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3034,7 +3042,7 @@
         <v>324</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="0"/>
@@ -3048,7 +3056,7 @@
         <v>85</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G29" s="6" t="str" cm="1">
         <f t="array" ref="G29">_xlfn.SWITCH(F29, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
@@ -3087,7 +3095,7 @@
         <v>325</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C30" t="str">
         <f t="shared" si="0"/>
@@ -3101,7 +3109,7 @@
         <v>85</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G30" s="6" t="str" cm="1">
         <f t="array" ref="G30">_xlfn.SWITCH(F30, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
@@ -3140,7 +3148,7 @@
         <v>326</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C31" t="str">
         <f t="shared" si="0"/>
@@ -3154,7 +3162,7 @@
         <v>85</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G31" s="6" t="str" cm="1">
         <f t="array" ref="G31">_xlfn.SWITCH(F31, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
@@ -3193,7 +3201,7 @@
         <v>327</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C32" t="str">
         <f t="shared" si="0"/>
@@ -3207,14 +3215,14 @@
         <v>85</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G32" s="6" t="str" cm="1">
         <f t="array" ref="G32">_xlfn.SWITCH(F32, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H32" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I32" t="s">
         <v>88</v>
@@ -3246,7 +3254,7 @@
         <v>328</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C33" t="str">
         <f t="shared" si="0"/>
@@ -3260,14 +3268,14 @@
         <v>85</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G33" s="6" t="str" cm="1">
         <f t="array" ref="G33">_xlfn.SWITCH(F33, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H33" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I33" t="s">
         <v>88</v>
@@ -3299,7 +3307,7 @@
         <v>329</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C34" t="str">
         <f t="shared" si="0"/>
@@ -3313,14 +3321,14 @@
         <v>85</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G34" s="6" t="str" cm="1">
         <f t="array" ref="G34">_xlfn.SWITCH(F34, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I34" t="s">
         <v>88</v>
@@ -3352,7 +3360,7 @@
         <v>330</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C35" t="str">
         <f t="shared" si="0"/>
@@ -3366,14 +3374,14 @@
         <v>85</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G35" s="6" t="str" cm="1">
         <f t="array" ref="G35">_xlfn.SWITCH(F35, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H35" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I35" t="s">
         <v>88</v>
@@ -3405,7 +3413,7 @@
         <v>331</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C36" t="str">
         <f t="shared" si="0"/>
@@ -3419,14 +3427,14 @@
         <v>85</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G36" s="6" t="str" cm="1">
         <f t="array" ref="G36">_xlfn.SWITCH(F36, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H36" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I36" t="s">
         <v>88</v>
@@ -4359,7 +4367,7 @@
         <v>801</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C54" t="str">
         <f t="shared" si="0"/>
@@ -4370,17 +4378,17 @@
         <v>Creamy Veggie Soup Recipe_Description</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>85</v>
+        <v>179</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G54" s="6" t="str" cm="1">
         <f t="array" ref="G54">_xlfn.SWITCH(F54, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="I54" t="s">
         <v>88</v>
@@ -4397,7 +4405,7 @@
         <v>802</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C55" t="str">
         <f t="shared" si="0"/>
@@ -4411,14 +4419,14 @@
         <v>85</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G55" s="6" t="str" cm="1">
         <f t="array" ref="G55">_xlfn.SWITCH(F55, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="I55" t="s">
         <v>88</v>
@@ -4435,7 +4443,7 @@
         <v>803</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" si="0"/>
@@ -4449,14 +4457,14 @@
         <v>85</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G56" s="6" t="str" cm="1">
         <f t="array" ref="G56">_xlfn.SWITCH(F56, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="I56" t="s">
         <v>88</v>
@@ -4473,7 +4481,7 @@
         <v>804</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C57" t="str">
         <f t="shared" si="0"/>
@@ -4487,14 +4495,14 @@
         <v>85</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G57" s="6" t="str" cm="1">
         <f t="array" ref="G57">_xlfn.SWITCH(F57, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="I57" t="s">
         <v>88</v>
@@ -4511,7 +4519,7 @@
         <v>805</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C58" t="str">
         <f t="shared" si="0"/>
@@ -4525,14 +4533,14 @@
         <v>85</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G58" s="6" t="str" cm="1">
         <f t="array" ref="G58">_xlfn.SWITCH(F58, "Resource", "#406672", "Animal Product", "#FF0064", "Vegetable", "#FF0064", "Fruit","#FF1493","Flower", "#DB36D3","Forage", "#0A8232","Recipe", "#DC3C00","Fish", "#00008B","Seed", "#A52A2A","Crafting", "#943D28","Mineral", "#6E005A", "Trash", "#696969","BASIC", "#313131","Tool", "#313131","Artisan Goods", "#009B6F", "Cooking", "#DC3C00","미지정")</f>
         <v>#DC3C00</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="I58" t="s">
         <v>88</v>
@@ -6575,7 +6583,7 @@
   <sheetData>
     <row r="3" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
@@ -6610,10 +6618,10 @@
         <v>153</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>154</v>
+        <v>181</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -6627,13 +6635,13 @@
         <v>801</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E5">
         <v>327</v>
@@ -6645,13 +6653,13 @@
         <v>802</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E6">
         <v>328</v>
@@ -6663,13 +6671,13 @@
         <v>803</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E7">
         <v>329</v>
@@ -6681,13 +6689,13 @@
         <v>804</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E8">
         <v>330</v>
@@ -6700,13 +6708,13 @@
         <v>805</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E9">
         <v>331</v>

</xml_diff>